<commit_message>
feat(F-NAR-019): TREE-AUT-039 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-039.xlsx
+++ b/stories/arbres/TREE-AUT-039.xlsx
@@ -2939,17 +2939,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le lièvre a le nez contre la poche. Nino porte la caisse, la corde à la paume. C'est moi le porteur, papa. Oui, elle est légère, maintenant. Le cube jaune garde un peu d'orange. Ils ont cherché dans la cuisine. La casserole tic, derrière eux. La rosée sèche sur le banc de mousse. Le chemin reprend, bas et clair.</t>
+          <t>Le lièvre a le nez contre la poche. Nino porte la caisse, la corde à la paume. C'est moi le porteur, papa. Oui, elle est légère, maintenant. Le cube jaune garde un peu d'orange. Ils ont cherché dans la cuisine. La casserole tic, derrière eux. La rosée sèche sur le banc de mousse. Nino avance, la caisse contre la hanche.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le lièvre a le nez contre la poche. Nino porte la caisse, la corde à la paume. C'est moi le porteur, papa. Oui, elle est légère, maintenant. Le cube jaune garde un peu d'orange. Ils ont cherché dans la cuisine. La casserole tic, derrière eux. La rosée sèche sur le banc de mousse. Le chemin reprend, bas et clair.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le lièvre a le nez contre la poche. Nino porte la caisse, la corde à la paume. C'est moi le porteur, papa. Oui, elle est légère, maintenant. Le cube jaune garde un peu d'orange. Ils ont cherché dans la cuisine. La casserole tic, derrière eux. La rosée sèche sur le banc de mousse. Nino avance, la caisse contre la hanche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le lièvre a le nez contre la poche. Nino porte la caisse, la corde à la paume. C'est moi le porteur, papa. Oui, elle est légère, maintenant. Le cube jaune garde un peu d'orange. Ils ont cherché dans la cuisine. La casserole tic, derrière eux. La rosée sèche sur le banc de mousse. Le chemin reprend, bas et clair.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le lièvre a le nez contre la poche. Nino porte la caisse, la corde à la paume. C'est moi le porteur, papa. Oui, elle est légère, maintenant. Le cube jaune garde un peu d'orange. Ils ont cherché dans la cuisine. La casserole tic, derrière eux. La rosée sèche sur le banc de mousse. Nino avance, la caisse contre la hanche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3091,7 +3091,7 @@
 narrateur|Ils ont cherché dans la cuisine.
 narrateur|La casserole tic, derrière eux.
 narrateur|La rosée sèche sur le banc de mousse.
-narrateur|Le chemin reprend, bas et clair.</t>
+narrateur|Nino avance, la caisse contre la hanche.</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Contre la joue, le lièvre est calme. Nino pose la caisse près de la grille. Les cubes font des ombres, dehors. La rue les a prises. Merci d'avoir porté jusqu'ici. L'ombre des cubes danse sous la lampe. La grille de cave est noire. Dehors, les lumières des maisons s'allument. L'osier ne cache plus rien.</t>
+          <t>Contre la joue, le lièvre est calme. Nino pose la caisse près de la grille. Les cubes font des ombres, dehors. La rue les a prises. Merci d'avoir porté jusqu'ici. L'ombre des cubes danse sous la lampe. La grille de cave est noire. Dehors, les lumières des maisons s'allument. La corde reste dans sa paume, sûre.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la joue, le lièvre est calme. Nino pose la caisse près de la grille. Les cubes font des ombres, dehors. La rue les a prises. Merci d'avoir porté jusqu'ici. L'ombre des cubes danse sous la lampe. La grille de cave est noire. Dehors, les lumières des maisons s'allument. L'osier ne cache plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la joue, le lièvre est calme. Nino pose la caisse près de la grille. Les cubes font des ombres, dehors. La rue les a prises. Merci d'avoir porté jusqu'ici. L'ombre des cubes danse sous la lampe. La grille de cave est noire. Dehors, les lumières des maisons s'allument. La corde reste dans sa paume, sûre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la joue, le lièvre est calme. Nino pose la caisse près de la grille. Les cubes font des ombres, dehors. La rue les a prises. Merci d'avoir porté jusqu'ici. L'ombre des cubes danse sous la lampe. La grille de cave est noire. Dehors, les lumières des maisons s'allument. L'osier ne cache plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la joue, le lièvre est calme. Nino pose la caisse près de la grille. Les cubes font des ombres, dehors. La rue les a prises. Merci d'avoir porté jusqu'ici. L'ombre des cubes danse sous la lampe. La grille de cave est noire. Dehors, les lumières des maisons s'allument. La corde reste dans sa paume, sûre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3833,7 +3833,7 @@
 narrateur|L'ombre des cubes danse sous la lampe.
 narrateur|La grille de cave est noire.
 narrateur|Dehors, les lumières des maisons s'allument.
-narrateur|L'osier ne cache plus rien.</t>
+narrateur|La corde reste dans sa paume, sûre.</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr">
@@ -6316,17 +6316,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Voilà le lièvre, contre le cartable. Nino pose la caisse sur le banc tiède. Il avait sa place à table. Au fond, oui. La cuillère a fini de briller. Une cuillère minuscule brille moins. Les joues de Nino sont chaudes. L'osier sent l'orange, un peu. Le banc garde leur poids.</t>
+          <t>Voilà le lièvre, contre le cartable. Nino pose la caisse sur le banc tiède. Il avait sa place à table. Au fond, oui. La cuillère a fini de briller. Une cuillère minuscule brille moins. Les joues de Nino sont chaudes. L'osier sent l'orange, un peu. La tasse miniature s'est tue, au fond.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Voilà le lièvre, contre le cartable. Nino pose la caisse sur le banc tiède. Il avait sa place à table. Au fond, oui. La cuillère a fini de briller. Une cuillère minuscule brille moins. Les joues de Nino sont chaudes. L'osier sent l'orange, un peu. Le banc garde leur poids.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Voilà le lièvre, contre le cartable. Nino pose la caisse sur le banc tiède. Il avait sa place à table. Au fond, oui. La cuillère a fini de briller. Une cuillère minuscule brille moins. Les joues de Nino sont chaudes. L'osier sent l'orange, un peu. La tasse miniature s'est tue, au fond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Voilà le lièvre, contre le cartable. Nino pose la caisse sur le banc tiède. Il avait sa place à table. Au fond, oui. La cuillère a fini de briller. Une cuillère minuscule brille moins. Les joues de Nino sont chaudes. L'osier sent l'orange, un peu. Le banc garde leur poids.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Voilà le lièvre, contre le cartable. Nino pose la caisse sur le banc tiède. Il avait sa place à table. Au fond, oui. La cuillère a fini de briller. Une cuillère minuscule brille moins. Les joues de Nino sont chaudes. L'osier sent l'orange, un peu. La tasse miniature s'est tue, au fond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6468,7 +6468,7 @@
 narrateur|Une cuillère minuscule brille moins.
 narrateur|Les joues de Nino sont chaudes.
 narrateur|L'osier sent l'orange, un peu.
-narrateur|Le banc garde leur poids.</t>
+narrateur|La tasse miniature s'est tue, au fond.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr">
@@ -9704,17 +9704,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Une goutte d'herbe sèche sur l'oreille. Nino porte la caisse, le livre au fond. La page est fraîche. Le chemin aussi. Le cartable te rejoint. Le livre a une page un peu fraîche. La rosée sèche sur le banc de mousse. Le moineau s'est envolé. Les pas reprennent, clairs.</t>
+          <t>Une goutte d'herbe sèche sur l'oreille. Nino porte la caisse, le livre au fond. La page est fraîche. Le chemin aussi. Le cartable te rejoint. Le livre a une page un peu fraîche. La rosée sèche sur le banc de mousse. Le moineau s'est envolé. Le livre frais tape le fond, au rythme des pas.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une goutte d'herbe sèche sur l'oreille. Nino porte la caisse, le livre au fond. La page est fraîche. Le chemin aussi. Le cartable te rejoint. Le livre a une page un peu fraîche. La rosée sèche sur le banc de mousse. Le moineau s'est envolé. Les pas reprennent, clairs.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une goutte d'herbe sèche sur l'oreille. Nino porte la caisse, le livre au fond. La page est fraîche. Le chemin aussi. Le cartable te rejoint. Le livre a une page un peu fraîche. La rosée sèche sur le banc de mousse. Le moineau s'est envolé. Le livre frais tape le fond, au rythme des pas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une goutte d'herbe sèche sur l'oreille. Nino porte la caisse, le livre au fond. La page est fraîche. Le chemin aussi. Le cartable te rejoint. Le livre a une page un peu fraîche. La rosée sèche sur le banc de mousse. Le moineau s'est envolé. Les pas reprennent, clairs.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une goutte d'herbe sèche sur l'oreille. Nino porte la caisse, le livre au fond. La page est fraîche. Le chemin aussi. Le cartable te rejoint. Le livre a une page un peu fraîche. La rosée sèche sur le banc de mousse. Le moineau s'est envolé. Le livre frais tape le fond, au rythme des pas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9856,7 +9856,7 @@
 narrateur|Le livre a une page un peu fraîche.
 narrateur|La rosée sèche sur le banc de mousse.
 narrateur|Le moineau s'est envolé.
-narrateur|Les pas reprennent, clairs.</t>
+narrateur|Le livre frais tape le fond, au rythme des pas.</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr">
@@ -11578,17 +11578,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Dans la paume, le bois est un peu frais. Nino pose la caisse sur le banc tiède. Son thé a attendu. Toi aussi. La cuillère est moins froide. L'osier sent le jardin tiède. Les joues de Nino restent chaudes. Une feuille reste dans l'assiette. Le banc garde leur poids.</t>
+          <t>Dans la paume, le bois est un peu frais. Nino pose la caisse sur le banc tiède. Son thé a attendu. Toi aussi. La cuillère est moins froide. L'osier sent le jardin tiède. Les joues de Nino restent chaudes. Une feuille reste dans l'assiette. L'herbe lâche leurs chaussures, enfin.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans la paume, le bois est un peu frais. Nino pose la caisse sur le banc tiède. Son thé a attendu. Toi aussi. La cuillère est moins froide. L'osier sent le jardin tiède. Les joues de Nino restent chaudes. Une feuille reste dans l'assiette. Le banc garde leur poids.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans la paume, le bois est un peu frais. Nino pose la caisse sur le banc tiède. Son thé a attendu. Toi aussi. La cuillère est moins froide. L'osier sent le jardin tiède. Les joues de Nino restent chaudes. Une feuille reste dans l'assiette. L'herbe lâche leurs chaussures, enfin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans la paume, le bois est un peu frais. Nino pose la caisse sur le banc tiède. Son thé a attendu. Toi aussi. La cuillère est moins froide. L'osier sent le jardin tiède. Les joues de Nino restent chaudes. Une feuille reste dans l'assiette. Le banc garde leur poids.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans la paume, le bois est un peu frais. Nino pose la caisse sur le banc tiède. Son thé a attendu. Toi aussi. La cuillère est moins froide. L'osier sent le jardin tiède. Les joues de Nino restent chaudes. Une feuille reste dans l'assiette. L'herbe lâche leurs chaussures, enfin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11730,7 +11730,7 @@
 narrateur|L'osier sent le jardin tiède.
 narrateur|Les joues de Nino restent chaudes.
 narrateur|Une feuille reste dans l'assiette.
-narrateur|Le banc garde leur poids.</t>
+narrateur|L'herbe lâche leurs chaussures, enfin.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
@@ -11949,17 +11949,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Nino souffle sur l'oreille du lièvre. L'assiette garde un rond de lampe. C'est son soleil. La rue en a un, trop. Passe, je ferme le pas. La petite assiette reflète le réverbère. La grille de cave est noire. Les maisons s'allument. Nino pose la caisse derrière la porte.</t>
+          <t>Nino souffle sur l'oreille du lièvre. L'assiette garde un rond de lampe. C'est son soleil. La rue a le sien, jaune. Passe, je ferme le pas. La petite assiette reflète le réverbère. La grille de cave est noire. Les maisons s'allument. Nino pose la caisse derrière la porte.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino souffle sur l'oreille du lièvre. L'assiette garde un rond de lampe. C'est son soleil. La rue en a un, trop. Passe, je ferme le pas. La petite assiette reflète le réverbère. La grille de cave est noire. Les maisons s'allument. Nino pose la caisse derrière la porte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino souffle sur l'oreille du lièvre. L'assiette garde un rond de lampe. C'est son soleil. La rue a le sien, jaune. Passe, je ferme le pas. La petite assiette reflète le réverbère. La grille de cave est noire. Les maisons s'allument. Nino pose la caisse derrière la porte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino souffle sur l'oreille du lièvre. L'assiette garde un rond de lampe. C'est son soleil. La rue en a un, trop. Passe, je ferme le pas. La petite assiette reflète le réverbère. La grille de cave est noire. Les maisons s'allument. Nino pose la caisse derrière la porte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino souffle sur l'oreille du lièvre. L'assiette garde un rond de lampe. C'est son soleil. La rue a le sien, jaune. Passe, je ferme le pas. La petite assiette reflète le réverbère. La grille de cave est noire. Les maisons s'allument. Nino pose la caisse derrière la porte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12096,7 +12096,7 @@
           <t>narrateur|Nino souffle sur l'oreille du lièvre.
 narrateur|L'assiette garde un rond de lampe.
 enfant-m|C'est son soleil.
-papa|La rue en a un, trop.
+papa|La rue a le sien, jaune.
 maman|Passe, je ferme le pas.
 narrateur|La petite assiette reflète le réverbère.
 narrateur|La grille de cave est noire.
@@ -13277,17 +13277,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>La lumière est pâle, un peu bleue. Nino glisse les cubes, un par un. Un cube tapote le parquet. Au fond, l'oreille de bois. Le chemin l'a mené là. Le vrai chemin, c'était l'osier. Le cartable est contre la chaise. Nino met le lièvre dans la poche. Il porte la caisse vers la porte. Le bonnet rejoint sa tête. La rosée sèche sur le banc. Le rideau jaune ne le retient plus.</t>
+          <t>La lumière est pâle, un peu bleue. Nino glisse les cubes, un par un. Un cube tapote le parquet. Au fond, l'oreille de bois. Le chemin l'a mené là. Il était au fond, Nino. Le cartable est contre la chaise. Nino met le lièvre dans la poche. Il porte la caisse vers la porte. Le bonnet rejoint sa tête. La rosée sèche sur le banc. Le rideau jaune ne le retient plus.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La lumière est pâle, un peu bleue. Nino glisse les cubes, un par un. Un cube tapote le parquet. Au fond, l'oreille de bois. Le chemin l'a mené là. Le vrai chemin, c'était l'osier. Le cartable est contre la chaise. Nino met le &lt;emphasis level="moderate"&gt;lièvre&lt;/emphasis&gt; dans la poche. Il porte la caisse vers la porte. Le bonnet rejoint sa tête. La rosée sèche sur le banc. Le rideau jaune ne le retient plus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La lumière est pâle, un peu bleue. Nino glisse les cubes, un par un. Un cube tapote le parquet. Au fond, l'oreille de bois. Le chemin l'a mené là. Il était au fond, Nino. Le cartable est contre la chaise. Nino met le &lt;emphasis level="moderate"&gt;lièvre&lt;/emphasis&gt; dans la poche. Il porte la caisse vers la porte. Le bonnet rejoint sa tête. La rosée sèche sur le banc. Le rideau jaune ne le retient plus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>La lumière est pâle, un peu bleue. Nino glisse les cubes, un par un. Un cube tapote le parquet. Au fond, l'oreille de bois. Le chemin l'a mené là. Le vrai chemin, c'était l'osier. Le cartable est contre la chaise. Nino met le &lt;emphasis&gt;lièvre&lt;/emphasis&gt; dans la poche. Il porte la caisse vers la porte. Le bonnet rejoint sa tête. La rosée sèche sur le banc. Le rideau jaune ne le retient plus. [pause]</t>
+          <t>La lumière est pâle, un peu bleue. Nino glisse les cubes, un par un. Un cube tapote le parquet. Au fond, l'oreille de bois. Le chemin l'a mené là. Il était au fond, Nino. Le cartable est contre la chaise. Nino met le &lt;emphasis&gt;lièvre&lt;/emphasis&gt; dans la poche. Il porte la caisse vers la porte. Le bonnet rejoint sa tête. La rosée sèche sur le banc. Le rideau jaune ne le retient plus. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13426,7 +13426,7 @@
 narrateur|Un cube tapote le parquet.
 narrateur|Au fond, l'oreille de bois.
 enfant-m|Le chemin l'a mené là.
-maman|Le vrai chemin, c'était l'osier.
+maman|Il était au fond, Nino.
 papa|Le cartable est contre la chaise.
 narrateur|Nino met le lièvre dans la poche.
 narrateur|Il porte la caisse vers la porte.
@@ -13464,17 +13464,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le cartable attend, sage, à côté. Nino porte la caisse, les cubes au fond. Le chemin de cubes est fini. Le vrai chemin est dehors. Le bonnet est sur ta tête. Un cube tapote le fond, très bas. La rosée sèche sur le banc de mousse. Le rideau jaune reste derrière. Les pas reprennent, clairs.</t>
+          <t>Le cartable attend, sage, à côté. Nino porte la caisse, les cubes au fond. Le chemin de cubes est fini. Dehors, le banc t'attend. Le bonnet est sur ta tête. Un cube tapote le fond, très bas. La rosée sèche sur le banc de mousse. Le rideau jaune reste derrière. Un cube tapote au rythme des pas.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable attend, sage, à côté. Nino porte la caisse, les cubes au fond. Le chemin de cubes est fini. Le vrai chemin est dehors. Le bonnet est sur ta tête. Un cube tapote le fond, très bas. La rosée sèche sur le banc de mousse. Le rideau jaune reste derrière. Les pas reprennent, clairs.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable attend, sage, à côté. Nino porte la caisse, les cubes au fond. Le chemin de cubes est fini. Dehors, le banc t'attend. Le bonnet est sur ta tête. Un cube tapote le fond, très bas. La rosée sèche sur le banc de mousse. Le rideau jaune reste derrière. Un cube tapote au rythme des pas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable attend, sage, à côté. Nino porte la caisse, les cubes au fond. Le chemin de cubes est fini. Le vrai chemin est dehors. Le bonnet est sur ta tête. Un cube tapote le fond, très bas. La rosée sèche sur le banc de mousse. Le rideau jaune reste derrière. Les pas reprennent, clairs.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable attend, sage, à côté. Nino porte la caisse, les cubes au fond. Le chemin de cubes est fini. Dehors, le banc t'attend. Le bonnet est sur ta tête. Un cube tapote le fond, très bas. La rosée sèche sur le banc de mousse. Le rideau jaune reste derrière. Un cube tapote au rythme des pas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13611,12 +13611,12 @@
           <t>narrateur|Le cartable attend, sage, à côté.
 narrateur|Nino porte la caisse, les cubes au fond.
 enfant-m|Le chemin de cubes est fini.
-papa|Le vrai chemin est dehors.
+papa|Dehors, le banc t'attend.
 maman|Le bonnet est sur ta tête.
 narrateur|Un cube tapote le fond, très bas.
 narrateur|La rosée sèche sur le banc de mousse.
 narrateur|Le rideau jaune reste derrière.
-narrateur|Les pas reprennent, clairs.</t>
+narrateur|Un cube tapote au rythme des pas.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr">
@@ -14206,17 +14206,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Le lièvre a un grain de lumière. Nino porte la caisse dans le couloir. Les cubes dansaient sur le mur. La veilleuse les a pris. La rue s'allume, elle aussi. L'ombre des cubes danse sur le mur. Les maisons, dehors, s'allument. La chambre garde un carré de veilleuse. L'osier ne cache plus rien.</t>
+          <t>Le lièvre a un grain de lumière. Nino porte la caisse dans le couloir. Les cubes dansaient sur le mur. La veilleuse les a pris. La rue s'allume, elle aussi. L'ombre des cubes danse sur le mur. Les maisons, dehors, s'allument. La chambre garde un carré de veilleuse. Le couloir sent le foin, un instant.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le lièvre a un grain de lumière. Nino porte la caisse dans le couloir. Les cubes dansaient sur le mur. La veilleuse les a pris. La rue s'allume, elle aussi. L'ombre des cubes danse sur le mur. Les maisons, dehors, s'allument. La chambre garde un carré de veilleuse. L'osier ne cache plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le lièvre a un grain de lumière. Nino porte la caisse dans le couloir. Les cubes dansaient sur le mur. La veilleuse les a pris. La rue s'allume, elle aussi. L'ombre des cubes danse sur le mur. Les maisons, dehors, s'allument. La chambre garde un carré de veilleuse. Le couloir sent le foin, un instant.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le lièvre a un grain de lumière. Nino porte la caisse dans le couloir. Les cubes dansaient sur le mur. La veilleuse les a pris. La rue s'allume, elle aussi. L'ombre des cubes danse sur le mur. Les maisons, dehors, s'allument. La chambre garde un carré de veilleuse. L'osier ne cache plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le lièvre a un grain de lumière. Nino porte la caisse dans le couloir. Les cubes dansaient sur le mur. La veilleuse les a pris. La rue s'allume, elle aussi. L'ombre des cubes danse sur le mur. Les maisons, dehors, s'allument. La chambre garde un carré de veilleuse. Le couloir sent le foin, un instant.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14358,7 +14358,7 @@
 narrateur|L'ombre des cubes danse sur le mur.
 narrateur|Les maisons, dehors, s'allument.
 narrateur|La chambre garde un carré de veilleuse.
-narrateur|L'osier ne cache plus rien.</t>
+narrateur|Le couloir sent le foin, un instant.</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr">
@@ -14967,17 +14967,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Nino referme la main autour du bois. Il porte la caisse, le livre au fond. Le rideau a laissé du jaune. Sur la page, oui. Le banc t'attend. Une bande jaune colore la page. La rosée sèche sur le banc de pierre. Le cartable fait zzz. Le chemin reprend, bas et clair.</t>
+          <t>Nino referme la main autour du bois. Il porte la caisse, le livre au fond. Le rideau a laissé du jaune. Sur la page, oui. Le banc t'attend. Une bande jaune colore la page. La rosée sèche sur le banc de pierre. Le cartable fait zzz. La bande jaune voyage avec la page.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino referme la main autour du bois. Il porte la caisse, le livre au fond. Le rideau a laissé du jaune. Sur la page, oui. Le banc t'attend. Une bande jaune colore la page. La rosée sèche sur le banc de pierre. Le cartable fait zzz. Le chemin reprend, bas et clair.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino referme la main autour du bois. Il porte la caisse, le livre au fond. Le rideau a laissé du jaune. Sur la page, oui. Le banc t'attend. Une bande jaune colore la page. La rosée sèche sur le banc de pierre. Le cartable fait zzz. La bande jaune voyage avec la page.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino referme la main autour du bois. Il porte la caisse, le livre au fond. Le rideau a laissé du jaune. Sur la page, oui. Le banc t'attend. Une bande jaune colore la page. La rosée sèche sur le banc de pierre. Le cartable fait zzz. Le chemin reprend, bas et clair.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino referme la main autour du bois. Il porte la caisse, le livre au fond. Le rideau a laissé du jaune. Sur la page, oui. Le banc t'attend. Une bande jaune colore la page. La rosée sèche sur le banc de pierre. Le cartable fait zzz. La bande jaune voyage avec la page.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15119,7 +15119,7 @@
 narrateur|Une bande jaune colore la page.
 narrateur|La rosée sèche sur le banc de pierre.
 narrateur|Le cartable fait zzz.
-narrateur|Le chemin reprend, bas et clair.</t>
+narrateur|La bande jaune voyage avec la page.</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr">
@@ -16470,17 +16470,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Nino a le bois contre le cœur. Il porte la caisse, la tasse au fond. Le thé de chambre est fini. Le chemin, lui, commence. Le cartable fait zzz. Une tasse miniature est au fond. La rosée sèche sur le banc de mousse. La fermeture du cartable se tait. Les pas reprennent, clairs.</t>
+          <t>Nino a le bois contre le cœur. Il porte la caisse, la tasse au fond. Le thé de chambre est fini. Le chemin, lui, commence. Le cartable fait zzz. Une tasse miniature est au fond. La rosée sèche sur le banc de mousse. Zzz, le cartable se tait. Sans ting, la tasse voyage au fond.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a le bois contre le cœur. Il porte la caisse, la tasse au fond. Le thé de chambre est fini. Le chemin, lui, commence. Le cartable fait zzz. Une tasse miniature est au fond. La rosée sèche sur le banc de mousse. La fermeture du cartable se tait. Les pas reprennent, clairs.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a le bois contre le cœur. Il porte la caisse, la tasse au fond. Le thé de chambre est fini. Le chemin, lui, commence. Le cartable fait zzz. Une tasse miniature est au fond. La rosée sèche sur le banc de mousse. Zzz, le cartable se tait. Sans ting, la tasse voyage au fond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a le bois contre le cœur. Il porte la caisse, la tasse au fond. Le thé de chambre est fini. Le chemin, lui, commence. Le cartable fait zzz. Une tasse miniature est au fond. La rosée sèche sur le banc de mousse. La fermeture du cartable se tait. Les pas reprennent, clairs.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a le bois contre le cœur. Il porte la caisse, la tasse au fond. Le thé de chambre est fini. Le chemin, lui, commence. Le cartable fait zzz. Une tasse miniature est au fond. La rosée sèche sur le banc de mousse. Zzz, le cartable se tait. Sans ting, la tasse voyage au fond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16621,8 +16621,8 @@
 papa|Le cartable fait zzz.
 narrateur|Une tasse miniature est au fond.
 narrateur|La rosée sèche sur le banc de mousse.
-narrateur|La fermeture du cartable se tait.
-narrateur|Les pas reprennent, clairs.</t>
+narrateur|Zzz, le cartable se tait.
+narrateur|Sans ting, la tasse voyage au fond.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -17390,7 +17390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17447,6 +17447,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>